<commit_message>
feat: simplify user-facing workbook
</commit_message>
<xml_diff>
--- a/examples/demo-labor-dispute/result-sample/案件材料汇总.xlsx
+++ b/examples/demo-labor-dispute/result-sample/案件材料汇总.xlsx
@@ -7,20 +7,20 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="案件链路总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文件清单" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体信息" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="音视频核对" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="时间轴" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="冲突与待核" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="案件概览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料清单" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当事人信息" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="音视频材料" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="案件时间轴" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题与待补材料" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'案件链路总览'!$A$3:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'文件清单'!$A$3:$K$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'主体信息'!$A$3:$J$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'音视频核对'!$A$3:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'时间轴'!$A$3:$M$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'冲突与待核'!$A$3:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'案件概览'!$A$3:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'材料清单'!$A$3:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'当事人信息'!$A$3:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'音视频材料'!$A$3:$D$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'案件时间轴'!$A$3:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'问题与待补材料'!$A$3:$D$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,25 +475,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>案件链路总览</t>
+          <t>案件概览</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>蓝色示例行仅说明填写格式，生成正式结果时删除；不确定内容填写“待核”，不得猜测。</t>
+          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
@@ -505,12 +504,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>内容</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>依据/事件编号</t>
+          <t>核心内容</t>
         </is>
       </c>
     </row>
@@ -525,11 +519,6 @@
           <t>材料显示，多家企业围绕南港医药物流园A区形成仓配及用工安排，员工陆续入场，但责任主体口径仍需核对。</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>待补充事件编号和材料编号</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -542,11 +531,6 @@
           <t>材料依次反映林晚晴盘点加班、孙浩现场事故及就医、高雪工资扣款等事项。</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>待补充事件编号和材料编号</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -559,11 +543,6 @@
           <t>争议集中在责任主体、加班工资、工伤及医疗费用、考勤扣款和延期支付。</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>待补充事件编号和材料编号</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -576,11 +555,6 @@
           <t>截至2025年3月5日，公司说明部分工资和补贴顺延，但材料未显示所有争议已结清。</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>待补充事件编号和材料编号</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -593,17 +567,12 @@
           <t>仍缺原始考勤、排班、事故申报、工伤认定、扣款依据及完整银行流水。</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>待补充事件编号和材料编号</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:C8"/>
+  <autoFilter ref="A3:B8"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -615,686 +584,452 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>文件清单</t>
+          <t>材料清单</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>蓝色示例行仅说明填写格式，生成正式结果时删除；不确定内容填写“待核”，不得猜测。</t>
+          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>材料编号</t>
+          <t>日期</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>原始文件名</t>
+          <t>材料名称</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>原始路径</t>
+          <t>材料类型</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>标准文件名</t>
+          <t>主要内容</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>归档路径</t>
+          <t>所在文件夹</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>扩展名</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>SHA-256</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>解析状态</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>重复组</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>版本组</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>备注</t>
+          <t>处理状态</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>MAT-0001</t>
+          <t>2024-03-12</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>IMG_0312_晚晴聊天.png</t>
+          <t>240312-林晚晴_私聊_加班未结算.png</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>IMG_0312_晚晴聊天.png</t>
+          <t>图片</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>240312-林晚晴_私聊_加班未结算.png</t>
+          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/240312-林晚晴_私聊_加班未结算.png</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>.png</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>46dc3b2bdc95136cb1a0cc11c3adc29d1d589afb44b33e844b55edb3aeab65e7</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>OCR已复核</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>MAT-0002</t>
+          <t>2024-08-30</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Screenshot_高雪扣款.png</t>
+          <t>240830-高雪_私聊_工资扣款.png</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Screenshot_高雪扣款.png</t>
+          <t>图片</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>240830-高雪_私聊_工资扣款.png</t>
+          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/240830-高雪_私聊_工资扣款.png</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>.png</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>9ca7030b0d370d9ca0a635462f3cfa90929bc300234942ae0553fad26be4f522</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>OCR已复核</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr"/>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>MAT-0003</t>
+          <t>2024-07-22</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>事故记录_孙浩.docx</t>
+          <t>240722-孙浩_现场事故记录.docx</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>事故记录_孙浩.docx</t>
+          <t>Word文档</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>240722-孙浩_现场事故记录.docx</t>
+          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/240722-孙浩_现场事故记录.docx</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>.docx</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>8d2d2d7a7344c152439cafa913c7e518ab8c0af9f96ed7521c5c5fcbdebf2b57</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>已提取</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="5" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>MAT-0004</t>
+          <t>2023-04-10</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>合同_晚晴_v2.docx</t>
+          <t>230410-林晚晴_E001_劳动合同.docx</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>合同_晚晴_v2.docx</t>
+          <t>合同</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>230410-林晚晴_E001_劳动合同.docx</t>
+          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/230410-林晚晴_E001_劳动合同.docx</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>.docx</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>56b91da0551dde1dd3f3f3f8b07b21baa4385aec87aec26c5284954845fdc092</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>已提取</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr"/>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>MAT-0005</t>
+          <t>2025-03-05</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>客户回款说明_最终版.txt</t>
+          <t>250305-工资支付延期说明.txt</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>客户回款说明_最终版.txt</t>
+          <t>文本材料</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>250305-工资支付延期说明.txt</t>
+          <t>延期说明称部分工资和补贴因客户结算延迟而顺延。</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/250305-工资支付延期说明.txt</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>.txt</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>5802d7a865469fb705b889ba91ca98e07e24d595e57cfe538dbe4412e50ab18d</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>已提取</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr"/>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>MAT-0006</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>工资条照片_3月.jpg</t>
+          <t>2403-林晚晴_工资条拍照件.jpg</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>工资条照片_3月.jpg</t>
+          <t>图片</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>2403-林晚晴_工资条拍照件.jpg</t>
+          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/2403-林晚晴_工资条拍照件.jpg</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>.jpg</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>a69d8b7e14da670c908fcdd901340689a875c87db644b24cda51ebbf488b514b</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>OCR已复核</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>MAT-0007</t>
+          <t>时间待确认</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>当事人情况汇总_未整理.txt</t>
+          <t>时间待核-案件当事人初始情况说明.txt</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>当事人情况汇总_未整理.txt</t>
+          <t>主体/工商材料</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>时间待核-案件当事人初始情况说明.txt</t>
+          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>001 主体信息/时间待核-案件当事人初始情况说明.txt</t>
+          <t>001 主体信息</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>.txt</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>76289b236ba59605190f301034cd4914f44b96ecef4efc74073c6e33a7ecae9e</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>已提取</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>MAT-0008</t>
+          <t>2023-03-06</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>总协议_扫描整理版.docx</t>
+          <t>230306-仓配服务与用工管理总协议.docx</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>总协议_扫描整理版.docx</t>
+          <t>协议</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>230306-仓配服务与用工管理总协议.docx</t>
+          <t>协议材料记载有关主体形成仓配服务和用工管理合作安排。</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/230306-仓配服务与用工管理总协议.docx</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>.docx</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>3c1495113075b11ab877e40a016ae83360aec622a90d2b6c80f85fcce11f7d4c</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>已提取</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>MAT-0009</t>
+          <t>2024-07-22</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>设备现场照片.jpg</t>
+          <t>240722-孙浩_现场设备照片.jpg</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>设备现场照片.jpg</t>
+          <t>图片/照片</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>240722-孙浩_现场设备照片.jpg</t>
+          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/240722-孙浩_现场设备照片.jpg</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>.jpg</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>ca3aa19b722bad0a2df65c3232d1337fc8a7277f39ad9818410f7b93d194a2b4</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>OCR已复核</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>MAT-0010</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>转账截图_晚晴.png</t>
+          <t>2403-林晚晴_银行转账详情.png</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>转账截图_晚晴.png</t>
+          <t>转账记录</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>2403-林晚晴_银行转账详情.png</t>
+          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/2403-林晚晴_银行转账详情.png</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>.png</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>d4438eb9d90c36b31720b17da4b85e9d2b44a7538a75e9bb7823b2762db94ba9</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>OCR已复核</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>MAT-0011</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>门诊票据_手机拍摄.jpg</t>
+          <t>240723-孙浩_门诊凭证照片.jpg</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>门诊票据_手机拍摄.jpg</t>
+          <t>图片/照片</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>240723-孙浩_门诊凭证照片.jpg</t>
+          <t>门诊凭证记载孙浩事故后就诊并发生医疗支出。</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/240723-孙浩_门诊凭证照片.jpg</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>.jpg</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>1bad183507ee827d2e991967384b0d2815c76ec4a6a696826cfc26b809e93118</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>OCR已复核</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr"/>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>MAT-0012</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>高雪工资条.jpg</t>
+          <t>2408-高雪_工资条拍照件.jpg</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>高雪工资条.jpg</t>
+          <t>图片</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>2408-高雪_工资条拍照件.jpg</t>
+          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料/2408-高雪_工资条拍照件.jpg</t>
+          <t>002 基础资料</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>.jpg</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>ac561d0725da3df87371b3497ea8fbf40ee48a3669b53d9bf5bb89e54aa69bd5</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>OCR已复核</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学示例；日期、主体和事件已经人工复核</t>
+          <t>已读取</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K15"/>
+  <autoFilter ref="A3:F15"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1306,134 +1041,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>主体信息</t>
+          <t>当事人信息</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>蓝色示例行仅说明填写格式，生成正式结果时删除；不确定内容填写“待核”，不得猜测。</t>
+          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>主体编号</t>
+          <t>姓名/公司</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>标准名称</t>
+          <t>身份或角色</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>主体类型</t>
+          <t>相关说明</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>别名</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>案件角色</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>强标识摘要</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>来源材料编号</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>原文定位</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>置信状态</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>待核事项</t>
+          <t>待确认事项</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>ENT-001</t>
+          <t>沪江优配仓储服务有限公司（演示）</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>沪江优配仓储服务有限公司（演示）</t>
+          <t>合同主体/管理主体候选</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>企业</t>
+          <t>类型：企业；其他称呼：沪江优配；用工单位；识别状态：中置信</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>沪江优配；用工单位</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>合同主体/管理主体候选</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>虚构教学主体</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0008；MAT-0004</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>协议和合同主体栏</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>发薪、社保和实际管理主体待核</t>
         </is>
@@ -1442,50 +1111,20 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>PER-001</t>
+          <t>林晚晴</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>林晚晴</t>
+          <t>员工/加班争议当事人</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>人员</t>
+          <t>类型：人员；其他称呼：晚晴；E001</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>晚晴；E001</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>员工/加班争议当事人</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>工号E001</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0004；MAT-0001</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>合同和聊天</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>无</t>
         </is>
@@ -1494,50 +1133,20 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>PER-002</t>
+          <t>孙浩</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>孙浩</t>
+          <t>员工/事故当事人</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>人员</t>
+          <t>类型：人员</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>员工/事故当事人</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>事故记录姓名</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0003；MAT-0011</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>事故记录和门诊凭证</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>工伤申报状态待核</t>
         </is>
@@ -1546,60 +1155,30 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>PER-003</t>
+          <t>高雪</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>高雪</t>
+          <t>员工/扣款争议当事人</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>人员</t>
+          <t>类型：人员</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>员工/扣款争议当事人</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>工资条姓名</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0012；MAT-0002</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>工资条和聊天</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
           <t>原始考勤待核</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J7"/>
+  <autoFilter ref="A3:D7"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1611,68 +1190,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>音视频核对</t>
+          <t>音视频材料</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>蓝色示例行仅说明填写格式，生成正式结果时删除；不确定内容填写“待核”，不得猜测。</t>
+          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>材料编号</t>
+          <t>文件名称</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>媒体文件</t>
+          <t>对应逐字稿</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>逐字稿文件</t>
+          <t>处理情况</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>匹配状态</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>是否纳入文本分析</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
           <t>备注</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F3"/>
+  <autoFilter ref="A3:D3"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1684,167 +1251,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>时间轴</t>
+          <t>案件时间轴</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>蓝色示例行仅说明填写格式，生成正式结果时删除；不确定内容填写“待核”，不得猜测。</t>
+          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>事件编号</t>
+          <t>日期</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>事件发生时间</t>
+          <t>事件</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>材料形成时间</t>
+          <t>相关人员/公司</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>时间精度</t>
+          <t>相关材料</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>地点/渠道</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>涉及主体</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>事件描述</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>主要材料编号</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>全部关联材料编号</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>原文定位</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>归档路径</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>记载性质</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>冲突/待核</t>
+          <t>待确认事项</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>EVT-001</t>
+          <t>2023-03-06</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2023-03-06</t>
+          <t>协议材料记载有关主体形成仓配服务和用工管理合作安排。</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>2023-03-06</t>
+          <t>沪江优配仓储服务有限公司（演示）等合作主体</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>230306-仓配服务与用工管理总协议.docx</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>南港医药物流园A区</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>沪江优配仓储服务有限公司（演示）等合作主体</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>协议材料记载有关主体形成仓配服务和用工管理合作安排。</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0008</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0008</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>协议主体和责任条款</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料/230306-仓配服务与用工管理总协议.docx</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>公司/书面记录</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>协议附件、盖章和具体责任边界仍待核。</t>
         </is>
@@ -1853,65 +1332,25 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>EVT-002</t>
+          <t>2023-04-10</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2023-04-10</t>
+          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>2023-04-10</t>
+          <t>林晚晴；沪江优配仓储服务有限公司（演示）</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>230410-林晚晴_E001_劳动合同.docx；时间待核-案件当事人初始情况说明.txt</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>A区仓库</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>林晚晴；沪江优配仓储服务有限公司（演示）</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0004</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0004；MAT-0007</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>合同基本信息；当事人情况汇总</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料/230410-林晚晴_E001_劳动合同.docx；001 主体信息/时间待核-案件当事人初始情况说明.txt</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>合同/人事记录</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>实际管理、发薪和社保主体需结合其他材料核对。</t>
         </is>
@@ -1920,65 +1359,25 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>EVT-003</t>
+          <t>2024-03-08至2024-03-10</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2024-03-08至2024-03-10</t>
+          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>2024-03至2024-03-12</t>
+          <t>林晚晴；现场主管</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>日期范围</t>
+          <t>240312-林晚晴_私聊_加班未结算.png；2403-林晚晴_工资条拍照件.jpg；2403-林晚晴_银行转账详情.png</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>A区仓库/企业聊天</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>林晚晴；现场主管</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0001</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0001；MAT-0006；MAT-0010</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>聊天截图；3月工资条；银行转账详情</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料/240312-林晚晴_私聊_加班未结算.png；002 基础资料/2403-林晚晴_工资条拍照件.jpg；002 基础资料/2403-林晚晴_银行转账详情.png</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>员工陈述+公司/系统记录</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>仍需原始考勤、排班和加班审批记录逐笔核对。</t>
         </is>
@@ -1987,65 +1386,25 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>EVT-004</t>
+          <t>2024-07-22</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2024-07-22</t>
+          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>2024-07-22</t>
+          <t>孙浩；现场主管</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>240722-孙浩_现场事故记录.docx；240722-孙浩_现场设备照片.jpg</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>A区2号输送线</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>孙浩；现场主管</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0003</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0003；MAT-0009</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>事故记录正文；设备现场照片</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料/240722-孙浩_现场事故记录.docx；002 基础资料/240722-孙浩_现场设备照片.jpg</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>公司记录+现场材料</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>设备状态、现场人员和事故申报情况待核。</t>
         </is>
@@ -2054,65 +1413,25 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>EVT-005</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>门诊凭证记载孙浩事故后就诊并发生医疗支出。</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>孙浩</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>240723-孙浩_门诊凭证照片.jpg</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>园区门诊</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>孙浩</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>门诊凭证记载孙浩事故后就诊并发生医疗支出。</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0011</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0011</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>门诊凭证照片</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料/240723-孙浩_门诊凭证照片.jpg</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>客观/医疗记录</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>票据原件、伤情和工伤关联性待核。</t>
         </is>
@@ -2121,65 +1440,25 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>EVT-006</t>
+          <t>2024-08-30</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>2024-08至2024-08-30</t>
+          <t>高雪；HR；财务</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>2408-高雪_工资条拍照件.jpg；240830-高雪_私聊_工资扣款.png</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>工资系统/企业聊天</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>高雪；HR；财务</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0012</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0012；MAT-0002</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>8月工资条；扣款沟通截图</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料/2408-高雪_工资条拍照件.jpg；002 基础资料/240830-高雪_私聊_工资扣款.png</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>公司记录+员工陈述</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>原始考勤、扣款计算和员工确认缺失。</t>
         </is>
@@ -2188,75 +1467,35 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>EVT-007</t>
+          <t>2025-03-05</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>2025-03-05</t>
+          <t>延期说明称部分工资和补贴因客户结算延迟而顺延。</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>2025-03-05</t>
+          <t>沪江优配仓储服务有限公司（演示）；相关员工</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>250305-工资支付延期说明.txt</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>公司说明</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>沪江优配仓储服务有限公司（演示）；相关员工</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>延期说明称部分工资和补贴因客户结算延迟而顺延。</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0005</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0005</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>说明文字</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料/250305-工资支付延期说明.txt</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>公司/书面记录</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
           <t>原说明、盖章状态和实际支付金额待核。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M10"/>
+  <autoFilter ref="A3:E10"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2268,101 +1507,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>冲突与待核</t>
+          <t>问题与待补材料</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>蓝色示例行仅说明填写格式，生成正式结果时删除；不确定内容填写“待核”，不得猜测。</t>
+          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>问题编号</t>
+          <t>问题</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>问题</t>
+          <t>可能影响</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>涉及事件</t>
+          <t>建议补充</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>涉及材料</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>可能影响</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>建议补充/核验</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>状态</t>
+          <t>处理状态</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>ISS-001</t>
+          <t>用工、管理、发薪和社保主体可能不一致</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>用工、管理、发薪和社保主体可能不一致</t>
+          <t>责任主体识别</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>EVT-001；EVT-002</t>
+          <t>补充工商、社保和银行流水记录</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0008；MAT-0004</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>责任主体识别</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>补充工商、社保和银行流水记录</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>待核</t>
         </is>
@@ -2371,35 +1577,20 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>ISS-002</t>
+          <t>盘点加班时长和支付金额未逐笔对应</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>盘点加班时长和支付金额未逐笔对应</t>
+          <t>加班工资计算</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>EVT-003</t>
+          <t>补充原始考勤、排班和审批</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0001；MAT-0006；MAT-0010</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>加班工资计算</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>补充原始考勤、排班和审批</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>待核</t>
         </is>
@@ -2408,35 +1599,20 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>ISS-003</t>
+          <t>事故申报及工伤认定材料缺失</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>事故申报及工伤认定材料缺失</t>
+          <t>工伤和医疗费用核验</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>EVT-004；EVT-005</t>
+          <t>补充事故申报、病历和认定材料</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0003；MAT-0011</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>工伤和医疗费用核验</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>补充事故申报、病历和认定材料</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>待核</t>
         </is>
@@ -2445,35 +1621,20 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>ISS-004</t>
+          <t>680元扣款缺少原始考勤和计算依据</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>680元扣款缺少原始考勤和计算依据</t>
+          <t>工资差额核验</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>EVT-006</t>
+          <t>调取原始考勤与扣款授权</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>MAT-0012；MAT-0002</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>工资差额核验</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>调取原始考勤与扣款授权</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>待核</t>
         </is>
@@ -2482,45 +1643,30 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>ISS-005</t>
+          <t>延期说明未显示争议已经结清</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>延期说明未显示争议已经结清</t>
+          <t>现状判断</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>EVT-007</t>
+          <t>以银行流水核对实际支付</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>MAT-0005</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>现状判断</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>以银行流水核对实际支付</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
           <t>待核</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G8"/>
+  <autoFilter ref="A3:D8"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>